<commit_message>
added some more stuff to the excel sheet
</commit_message>
<xml_diff>
--- a/assets/item_list.xlsx
+++ b/assets/item_list.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20361"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{864E927F-E2CB-4AF6-B17A-1D84A4719DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1543CE32-6A22-4704-9E8B-6E176328832D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11,7 +11,7 @@
     <sheet name="ItemList" sheetId="1" r:id="rId1"/>
     <sheet name="Notes" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="79">
   <si>
     <t>halberd</t>
   </si>
@@ -158,9 +158,6 @@
     <t>Item Type</t>
   </si>
   <si>
-    <t>Item Rarity</t>
-  </si>
-  <si>
     <t>Item ID</t>
   </si>
   <si>
@@ -185,9 +182,6 @@
     <t>Epic</t>
   </si>
   <si>
-    <t>Class Type</t>
-  </si>
-  <si>
     <t>*rarity 1 and class type 0 for now</t>
   </si>
   <si>
@@ -201,6 +195,69 @@
   </si>
   <si>
     <t>*default power and speed = 10 for now</t>
+  </si>
+  <si>
+    <t>Defense</t>
+  </si>
+  <si>
+    <t>No.</t>
+  </si>
+  <si>
+    <t>Class Type 1</t>
+  </si>
+  <si>
+    <t>Class Type 2</t>
+  </si>
+  <si>
+    <t>Item Class Set</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Z</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Demon</t>
+  </si>
+  <si>
+    <t>Fighter</t>
+  </si>
+  <si>
+    <t>fighter</t>
+  </si>
+  <si>
+    <t>archer</t>
+  </si>
+  <si>
+    <t>tank</t>
+  </si>
+  <si>
+    <t>beserker</t>
+  </si>
+  <si>
+    <t>wizard</t>
+  </si>
+  <si>
+    <t>assasin</t>
+  </si>
+  <si>
+    <t>demon</t>
+  </si>
+  <si>
+    <t>necromancer</t>
   </si>
 </sst>
 </file>
@@ -277,7 +334,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -295,6 +352,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -575,19 +635,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.140625" style="1" customWidth="1"/>
-    <col min="3" max="4" width="11.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="9.28515625" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" customWidth="1"/>
+    <col min="6" max="6" width="13" customWidth="1"/>
     <col min="7" max="7" width="9.85546875" customWidth="1"/>
+    <col min="8" max="8" width="12.140625" customWidth="1"/>
     <col min="12" max="12" width="14.85546875" customWidth="1"/>
     <col min="14" max="14" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>43</v>
       </c>
@@ -595,25 +658,43 @@
         <v>44</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="L1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -623,20 +704,33 @@
       <c r="C2" s="1">
         <v>1</v>
       </c>
-      <c r="D2" s="1">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>11001</v>
-      </c>
-      <c r="F2" s="1">
-        <v>10</v>
+      <c r="D2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" s="1">
+        <v>5</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="G2" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="I2" s="1"/>
+      <c r="J2">
+        <v>158</v>
+      </c>
+      <c r="K2" s="1">
+        <v>10</v>
+      </c>
+      <c r="L2" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -646,20 +740,33 @@
       <c r="C3" s="1">
         <v>1</v>
       </c>
-      <c r="D3" s="1">
-        <v>0</v>
-      </c>
-      <c r="E3">
+      <c r="D3" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G3" s="1">
+        <v>1</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I3" s="1"/>
+      <c r="J3">
         <v>11002</v>
       </c>
-      <c r="F3" s="1">
-        <v>10</v>
-      </c>
-      <c r="G3" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K3" s="1">
+        <v>10</v>
+      </c>
+      <c r="L3" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>31</v>
       </c>
@@ -669,20 +776,33 @@
       <c r="C4" s="1">
         <v>1</v>
       </c>
-      <c r="D4" s="1">
-        <v>0</v>
-      </c>
-      <c r="E4">
+      <c r="D4" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G4" s="1">
+        <v>1</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I4" s="1"/>
+      <c r="J4">
         <v>11003</v>
       </c>
-      <c r="F4" s="1">
-        <v>10</v>
-      </c>
-      <c r="G4" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K4" s="1">
+        <v>10</v>
+      </c>
+      <c r="L4" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>32</v>
       </c>
@@ -692,20 +812,33 @@
       <c r="C5" s="1">
         <v>1</v>
       </c>
-      <c r="D5" s="1">
-        <v>0</v>
-      </c>
-      <c r="E5">
+      <c r="D5" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E5" s="1">
+        <v>2</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="G5" s="1">
+        <v>1</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="I5" s="1"/>
+      <c r="J5">
         <v>11004</v>
       </c>
-      <c r="F5" s="1">
-        <v>10</v>
-      </c>
-      <c r="G5" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K5" s="1">
+        <v>10</v>
+      </c>
+      <c r="L5" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -715,20 +848,33 @@
       <c r="C6" s="1">
         <v>1</v>
       </c>
-      <c r="D6" s="1">
-        <v>0</v>
-      </c>
-      <c r="E6">
+      <c r="D6" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G6" s="1">
+        <v>2</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="I6" s="1"/>
+      <c r="J6">
         <v>11005</v>
       </c>
-      <c r="F6" s="1">
-        <v>10</v>
-      </c>
-      <c r="G6" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K6" s="1">
+        <v>10</v>
+      </c>
+      <c r="L6" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -738,20 +884,33 @@
       <c r="C7" s="1">
         <v>1</v>
       </c>
-      <c r="D7" s="1">
-        <v>0</v>
-      </c>
-      <c r="E7">
+      <c r="D7" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E7" s="1">
+        <v>2</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" s="1">
+        <v>2</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I7" s="1"/>
+      <c r="J7">
         <v>11006</v>
       </c>
-      <c r="F7" s="1">
-        <v>10</v>
-      </c>
-      <c r="G7" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K7" s="1">
+        <v>10</v>
+      </c>
+      <c r="L7" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -761,20 +920,33 @@
       <c r="C8" s="1">
         <v>1</v>
       </c>
-      <c r="D8" s="1">
-        <v>0</v>
-      </c>
-      <c r="E8">
+      <c r="D8" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" s="1">
+        <v>3</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G8" s="1">
+        <v>4</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="I8" s="1"/>
+      <c r="J8">
         <v>11007</v>
       </c>
-      <c r="F8" s="1">
-        <v>10</v>
-      </c>
-      <c r="G8" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K8" s="1">
+        <v>10</v>
+      </c>
+      <c r="L8" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -784,20 +956,33 @@
       <c r="C9" s="1">
         <v>1</v>
       </c>
-      <c r="D9" s="1">
-        <v>0</v>
-      </c>
-      <c r="E9">
+      <c r="D9" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" s="1">
+        <v>3</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G9" s="1">
+        <v>5</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="I9" s="1"/>
+      <c r="J9">
         <v>11008</v>
       </c>
-      <c r="F9" s="1">
-        <v>10</v>
-      </c>
-      <c r="G9" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K9" s="1">
+        <v>10</v>
+      </c>
+      <c r="L9" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>36</v>
       </c>
@@ -807,20 +992,33 @@
       <c r="C10" s="1">
         <v>1</v>
       </c>
-      <c r="D10" s="1">
-        <v>0</v>
-      </c>
-      <c r="E10">
+      <c r="D10" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="1">
+        <v>5</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G10" s="1">
+        <v>5</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="I10" s="1"/>
+      <c r="J10">
         <v>11009</v>
       </c>
-      <c r="F10" s="1">
-        <v>10</v>
-      </c>
-      <c r="G10" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K10" s="1">
+        <v>10</v>
+      </c>
+      <c r="L10" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>1</v>
       </c>
@@ -830,20 +1028,33 @@
       <c r="C11" s="1">
         <v>1</v>
       </c>
-      <c r="D11" s="1">
-        <v>0</v>
-      </c>
-      <c r="E11">
+      <c r="D11" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" s="1">
+        <v>4</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G11" s="1">
+        <v>6</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="I11" s="1"/>
+      <c r="J11">
         <v>11010</v>
       </c>
-      <c r="F11" s="1">
-        <v>10</v>
-      </c>
-      <c r="G11" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K11" s="1">
+        <v>10</v>
+      </c>
+      <c r="L11" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>37</v>
       </c>
@@ -853,20 +1064,33 @@
       <c r="C12" s="1">
         <v>1</v>
       </c>
-      <c r="D12" s="1">
-        <v>0</v>
-      </c>
-      <c r="E12">
+      <c r="D12" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E12" s="1">
+        <v>2</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G12" s="1">
+        <v>3</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I12" s="1"/>
+      <c r="J12">
         <v>11011</v>
       </c>
-      <c r="F12" s="1">
-        <v>10</v>
-      </c>
-      <c r="G12" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K12" s="1">
+        <v>10</v>
+      </c>
+      <c r="L12" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>38</v>
       </c>
@@ -876,20 +1100,33 @@
       <c r="C13" s="1">
         <v>1</v>
       </c>
-      <c r="D13" s="1">
-        <v>0</v>
-      </c>
-      <c r="E13">
+      <c r="D13" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E13" s="1">
+        <v>3</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G13" s="1">
+        <v>3</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="I13" s="1"/>
+      <c r="J13">
         <v>11012</v>
       </c>
-      <c r="F13" s="1">
-        <v>10</v>
-      </c>
-      <c r="G13" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K13" s="1">
+        <v>10</v>
+      </c>
+      <c r="L13" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>39</v>
       </c>
@@ -899,20 +1136,33 @@
       <c r="C14" s="1">
         <v>1</v>
       </c>
-      <c r="D14" s="1">
-        <v>0</v>
-      </c>
-      <c r="E14">
+      <c r="D14" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E14" s="1">
+        <v>1</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G14" s="1">
+        <v>7</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="I14" s="1"/>
+      <c r="J14">
         <v>11013</v>
       </c>
-      <c r="F14" s="1">
-        <v>10</v>
-      </c>
-      <c r="G14" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K14" s="1">
+        <v>10</v>
+      </c>
+      <c r="L14" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>40</v>
       </c>
@@ -922,20 +1172,33 @@
       <c r="C15" s="1">
         <v>1</v>
       </c>
-      <c r="D15" s="1">
-        <v>0</v>
-      </c>
-      <c r="E15">
+      <c r="D15" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" s="1">
+        <v>2</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G15" s="1">
+        <v>7</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I15" s="1"/>
+      <c r="J15">
         <v>11014</v>
       </c>
-      <c r="F15" s="1">
-        <v>10</v>
-      </c>
-      <c r="G15" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K15" s="1">
+        <v>10</v>
+      </c>
+      <c r="L15" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>41</v>
       </c>
@@ -945,20 +1208,33 @@
       <c r="C16" s="1">
         <v>1</v>
       </c>
-      <c r="D16" s="1">
-        <v>0</v>
-      </c>
-      <c r="E16">
+      <c r="D16" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E16" s="1">
+        <v>4</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="1">
+        <v>8</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="I16" s="1"/>
+      <c r="J16">
         <v>11015</v>
       </c>
-      <c r="F16" s="1">
-        <v>10</v>
-      </c>
-      <c r="G16" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="K16" s="1">
+        <v>10</v>
+      </c>
+      <c r="L16" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>3</v>
       </c>
@@ -968,20 +1244,31 @@
       <c r="C17" s="1">
         <v>1</v>
       </c>
-      <c r="D17" s="1">
-        <v>0</v>
-      </c>
-      <c r="E17">
+      <c r="D17" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E17" s="1">
+        <v>4</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G17" s="1">
+        <v>5</v>
+      </c>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17">
         <v>11016</v>
       </c>
-      <c r="F17" s="1">
-        <v>10</v>
-      </c>
-      <c r="G17" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="K17" s="1">
+        <v>10</v>
+      </c>
+      <c r="L17" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>4</v>
       </c>
@@ -991,20 +1278,31 @@
       <c r="C18" s="1">
         <v>1</v>
       </c>
-      <c r="D18" s="1">
-        <v>0</v>
-      </c>
-      <c r="E18">
+      <c r="D18" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" s="1">
+        <v>1</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="G18" s="1">
+        <v>1</v>
+      </c>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18">
         <v>11017</v>
       </c>
-      <c r="F18" s="1">
-        <v>10</v>
-      </c>
-      <c r="G18" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="K18" s="1">
+        <v>10</v>
+      </c>
+      <c r="L18" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>29</v>
       </c>
@@ -1012,16 +1310,23 @@
         <v>28</v>
       </c>
       <c r="C19" s="1">
-        <v>1</v>
-      </c>
-      <c r="D19" s="1">
+        <v>2</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E19" s="1">
         <v>0</v>
       </c>
-      <c r="E19">
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19">
         <v>21001</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>13</v>
       </c>
@@ -1029,16 +1334,23 @@
         <v>28</v>
       </c>
       <c r="C20" s="1">
-        <v>1</v>
-      </c>
-      <c r="D20" s="1">
+        <v>2</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E20" s="1">
         <v>0</v>
       </c>
-      <c r="E20">
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20">
         <v>21002</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>14</v>
       </c>
@@ -1046,16 +1358,23 @@
         <v>28</v>
       </c>
       <c r="C21" s="1">
-        <v>1</v>
-      </c>
-      <c r="D21" s="1">
+        <v>2</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E21" s="1">
         <v>0</v>
       </c>
-      <c r="E21">
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21">
         <v>21003</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>15</v>
       </c>
@@ -1063,16 +1382,23 @@
         <v>28</v>
       </c>
       <c r="C22" s="1">
-        <v>1</v>
-      </c>
-      <c r="D22" s="1">
+        <v>2</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E22" s="1">
         <v>0</v>
       </c>
-      <c r="E22">
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22">
         <v>21004</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>16</v>
       </c>
@@ -1080,16 +1406,23 @@
         <v>28</v>
       </c>
       <c r="C23" s="1">
-        <v>1</v>
-      </c>
-      <c r="D23" s="1">
+        <v>2</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E23" s="1">
         <v>0</v>
       </c>
-      <c r="E23">
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23">
         <v>21005</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>17</v>
       </c>
@@ -1097,16 +1430,23 @@
         <v>28</v>
       </c>
       <c r="C24" s="1">
-        <v>1</v>
-      </c>
-      <c r="D24" s="1">
+        <v>2</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E24" s="1">
         <v>0</v>
       </c>
-      <c r="E24">
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24">
         <v>21006</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>18</v>
       </c>
@@ -1114,16 +1454,23 @@
         <v>28</v>
       </c>
       <c r="C25" s="1">
-        <v>1</v>
-      </c>
-      <c r="D25" s="1">
+        <v>2</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E25" s="1">
         <v>0</v>
       </c>
-      <c r="E25">
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25">
         <v>21007</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>19</v>
       </c>
@@ -1131,16 +1478,23 @@
         <v>28</v>
       </c>
       <c r="C26" s="1">
-        <v>1</v>
-      </c>
-      <c r="D26" s="1">
+        <v>2</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E26" s="1">
         <v>0</v>
       </c>
-      <c r="E26">
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26">
         <v>21008</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>20</v>
       </c>
@@ -1148,16 +1502,23 @@
         <v>28</v>
       </c>
       <c r="C27" s="1">
-        <v>1</v>
-      </c>
-      <c r="D27" s="1">
+        <v>2</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E27" s="1">
         <v>0</v>
       </c>
-      <c r="E27">
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27">
         <v>21009</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>21</v>
       </c>
@@ -1165,16 +1526,23 @@
         <v>28</v>
       </c>
       <c r="C28" s="1">
-        <v>1</v>
-      </c>
-      <c r="D28" s="1">
+        <v>2</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E28" s="1">
         <v>0</v>
       </c>
-      <c r="E28">
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28">
         <v>21010</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>22</v>
       </c>
@@ -1182,16 +1550,23 @@
         <v>28</v>
       </c>
       <c r="C29" s="1">
-        <v>1</v>
-      </c>
-      <c r="D29" s="1">
+        <v>2</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E29" s="1">
         <v>0</v>
       </c>
-      <c r="E29">
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29">
         <v>21011</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -1199,16 +1574,23 @@
         <v>28</v>
       </c>
       <c r="C30" s="1">
-        <v>1</v>
-      </c>
-      <c r="D30" s="1">
+        <v>2</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E30" s="1">
         <v>0</v>
       </c>
-      <c r="E30">
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30">
         <v>21012</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>24</v>
       </c>
@@ -1216,16 +1598,23 @@
         <v>28</v>
       </c>
       <c r="C31" s="1">
-        <v>1</v>
-      </c>
-      <c r="D31" s="1">
+        <v>2</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E31" s="1">
         <v>0</v>
       </c>
-      <c r="E31">
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31">
         <v>21013</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>25</v>
       </c>
@@ -1233,16 +1622,23 @@
         <v>28</v>
       </c>
       <c r="C32" s="1">
-        <v>1</v>
-      </c>
-      <c r="D32" s="1">
+        <v>2</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E32" s="1">
         <v>0</v>
       </c>
-      <c r="E32">
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32">
         <v>21014</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>26</v>
       </c>
@@ -1250,16 +1646,23 @@
         <v>28</v>
       </c>
       <c r="C33" s="1">
-        <v>1</v>
-      </c>
-      <c r="D33" s="1">
+        <v>2</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E33" s="1">
         <v>0</v>
       </c>
-      <c r="E33">
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33">
         <v>21015</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>27</v>
       </c>
@@ -1267,14 +1670,51 @@
         <v>28</v>
       </c>
       <c r="C34" s="1">
-        <v>1</v>
-      </c>
-      <c r="D34" s="1">
+        <v>2</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E34" s="1">
         <v>0</v>
       </c>
-      <c r="E34">
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34">
         <v>21016</v>
       </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E35" s="1"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E36" s="1"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E37" s="1"/>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E38" s="1"/>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E39" s="1"/>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E40" s="1"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E41" s="1"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E42" s="1"/>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E43" s="1"/>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E44" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1319,7 +1759,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D4" s="5">
         <v>1</v>
@@ -1333,7 +1773,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D5" s="5">
         <v>2</v>
@@ -1341,13 +1781,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6" s="5">
         <v>3</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D6" s="5">
         <v>3</v>
@@ -1355,13 +1795,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B7" s="5">
         <v>4</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D7" s="5">
         <v>4</v>
@@ -1369,7 +1809,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B8" s="5">
         <v>5</v>
@@ -1379,12 +1819,12 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
just added some more stuff to the excel sheet
</commit_message>
<xml_diff>
--- a/assets/item_list.xlsx
+++ b/assets/item_list.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20361"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1543CE32-6A22-4704-9E8B-6E176328832D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B1F75F8-BF87-43BC-9FAD-CADCC0932735}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="81">
   <si>
     <t>halberd</t>
   </si>
@@ -258,6 +258,12 @@
   </si>
   <si>
     <t>necromancer</t>
+  </si>
+  <si>
+    <t>ARMORS</t>
+  </si>
+  <si>
+    <t>WEAPONS</t>
   </si>
 </sst>
 </file>
@@ -334,7 +340,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -355,6 +361,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -635,7 +649,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:O48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" customWidth="1"/>
@@ -651,88 +665,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1"/>
+      <c r="F1"/>
+      <c r="G1"/>
+      <c r="H1"/>
+      <c r="I1"/>
+      <c r="J1"/>
+      <c r="K1"/>
+      <c r="L1"/>
+      <c r="M1"/>
+      <c r="N1"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>56</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="1">
-        <v>1</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="E2" s="1">
-        <v>5</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="G2" s="1">
-        <v>8</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="I2" s="1"/>
-      <c r="J2">
-        <v>158</v>
-      </c>
-      <c r="K2" s="1">
-        <v>10</v>
-      </c>
-      <c r="L2" s="1">
-        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>12</v>
@@ -741,23 +737,25 @@
         <v>1</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E3" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G3" s="1">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I3" s="1"/>
+        <v>74</v>
+      </c>
+      <c r="I3" s="1">
+        <v>5</v>
+      </c>
       <c r="J3">
-        <v>11002</v>
+        <v>1585</v>
       </c>
       <c r="K3" s="1">
         <v>10</v>
@@ -768,7 +766,7 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>12</v>
@@ -783,17 +781,19 @@
         <v>1</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="G4" s="1">
         <v>1</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I4" s="1"/>
+        <v>73</v>
+      </c>
+      <c r="I4" s="1">
+        <v>4</v>
+      </c>
       <c r="J4">
-        <v>11003</v>
+        <v>1114</v>
       </c>
       <c r="K4" s="1">
         <v>10</v>
@@ -804,7 +804,7 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>12</v>
@@ -813,23 +813,25 @@
         <v>1</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E5" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="G5" s="1">
         <v>1</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="I5" s="1"/>
+        <v>76</v>
+      </c>
+      <c r="I5" s="1">
+        <v>7</v>
+      </c>
       <c r="J5">
-        <v>11004</v>
+        <v>1117</v>
       </c>
       <c r="K5" s="1">
         <v>10</v>
@@ -840,7 +842,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>12</v>
@@ -849,23 +851,25 @@
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E6" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G6" s="1">
-        <v>2</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="I6" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="I6" s="1">
+        <v>8</v>
+      </c>
       <c r="J6">
-        <v>11005</v>
+        <v>1218</v>
       </c>
       <c r="K6" s="1">
         <v>10</v>
@@ -876,7 +880,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>12</v>
@@ -885,10 +889,10 @@
         <v>1</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E7" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>72</v>
@@ -896,12 +900,12 @@
       <c r="G7" s="1">
         <v>2</v>
       </c>
-      <c r="H7" s="1" t="s">
-        <v>75</v>
+      <c r="H7" s="9" t="s">
+        <v>68</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7">
-        <v>11006</v>
+        <v>1120</v>
       </c>
       <c r="K7" s="1">
         <v>10</v>
@@ -912,7 +916,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>12</v>
@@ -921,23 +925,25 @@
         <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E8" s="1">
+        <v>2</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G8" s="1">
+        <v>2</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I8" s="1">
         <v>3</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G8" s="1">
-        <v>4</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="I8" s="1"/>
       <c r="J8">
-        <v>11007</v>
+        <v>1223</v>
       </c>
       <c r="K8" s="1">
         <v>10</v>
@@ -948,7 +954,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>12</v>
@@ -963,17 +969,19 @@
         <v>3</v>
       </c>
       <c r="F9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G9" s="1">
+        <v>4</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="G9" s="1">
+      <c r="I9" s="1">
         <v>5</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="I9" s="1"/>
       <c r="J9">
-        <v>11008</v>
+        <v>1345</v>
       </c>
       <c r="K9" s="1">
         <v>10</v>
@@ -984,7 +992,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>12</v>
@@ -993,10 +1001,10 @@
         <v>1</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E10" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>74</v>
@@ -1005,11 +1013,13 @@
         <v>5</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="I10" s="1"/>
+        <v>71</v>
+      </c>
+      <c r="I10" s="1">
+        <v>1</v>
+      </c>
       <c r="J10">
-        <v>11009</v>
+        <v>1351</v>
       </c>
       <c r="K10" s="1">
         <v>10</v>
@@ -1020,7 +1030,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>12</v>
@@ -1029,23 +1039,25 @@
         <v>1</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E11" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G11" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="I11" s="1"/>
+      <c r="I11" s="1">
+        <v>8</v>
+      </c>
       <c r="J11">
-        <v>11010</v>
+        <v>1558</v>
       </c>
       <c r="K11" s="1">
         <v>10</v>
@@ -1056,7 +1068,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>12</v>
@@ -1065,23 +1077,25 @@
         <v>1</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E12" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G12" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="I12" s="1"/>
+        <v>77</v>
+      </c>
+      <c r="I12" s="1">
+        <v>8</v>
+      </c>
       <c r="J12">
-        <v>11011</v>
+        <v>1468</v>
       </c>
       <c r="K12" s="1">
         <v>10</v>
@@ -1092,7 +1106,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>12</v>
@@ -1101,10 +1115,10 @@
         <v>1</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E13" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>75</v>
@@ -1113,11 +1127,13 @@
         <v>3</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="I13" s="1"/>
+        <v>72</v>
+      </c>
+      <c r="I13" s="1">
+        <v>2</v>
+      </c>
       <c r="J13">
-        <v>11012</v>
+        <v>1232</v>
       </c>
       <c r="K13" s="1">
         <v>10</v>
@@ -1128,7 +1144,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>12</v>
@@ -1137,23 +1153,25 @@
         <v>1</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E14" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G14" s="1">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="I14" s="1"/>
+        <v>78</v>
+      </c>
+      <c r="I14" s="1">
+        <v>6</v>
+      </c>
       <c r="J14">
-        <v>11013</v>
+        <v>1336</v>
       </c>
       <c r="K14" s="1">
         <v>10</v>
@@ -1164,7 +1182,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>12</v>
@@ -1173,10 +1191,10 @@
         <v>1</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E15" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>76</v>
@@ -1185,11 +1203,13 @@
         <v>7</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="I15" s="1"/>
+        <v>71</v>
+      </c>
+      <c r="I15" s="1">
+        <v>1</v>
+      </c>
       <c r="J15">
-        <v>11014</v>
+        <v>1171</v>
       </c>
       <c r="K15" s="1">
         <v>10</v>
@@ -1200,7 +1220,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>12</v>
@@ -1209,23 +1229,25 @@
         <v>1</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E16" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G16" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="I16" s="1"/>
+        <v>72</v>
+      </c>
+      <c r="I16" s="1">
+        <v>2</v>
+      </c>
       <c r="J16">
-        <v>11015</v>
+        <v>1272</v>
       </c>
       <c r="K16" s="1">
         <v>10</v>
@@ -1234,9 +1256,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>12</v>
@@ -1251,15 +1273,17 @@
         <v>4</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="G17" s="1">
-        <v>5</v>
-      </c>
-      <c r="H17" s="1"/>
+        <v>8</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>68</v>
+      </c>
       <c r="I17" s="1"/>
       <c r="J17">
-        <v>11016</v>
+        <v>1480</v>
       </c>
       <c r="K17" s="1">
         <v>10</v>
@@ -1268,9 +1292,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>12</v>
@@ -1279,128 +1303,112 @@
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" s="1">
+        <v>4</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G18" s="1">
+        <v>5</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I18" s="1">
+        <v>4</v>
+      </c>
+      <c r="J18">
+        <v>1454</v>
+      </c>
+      <c r="K18" s="1">
+        <v>10</v>
+      </c>
+      <c r="L18" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="1">
+        <v>1</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E18" s="1">
-        <v>1</v>
-      </c>
-      <c r="F18" s="1" t="s">
+      <c r="E19" s="1">
+        <v>1</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="G18" s="1">
-        <v>1</v>
-      </c>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18">
-        <v>11017</v>
-      </c>
-      <c r="K18" s="1">
-        <v>10</v>
-      </c>
-      <c r="L18" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>29</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C19" s="1">
-        <v>2</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E19" s="1">
-        <v>0</v>
-      </c>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
+      <c r="G19" s="1">
+        <v>1</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I19" s="1">
+        <v>7</v>
+      </c>
       <c r="J19">
-        <v>21001</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>13</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C20" s="1">
-        <v>2</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E20" s="1">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K19" s="1">
+        <v>10</v>
+      </c>
+      <c r="L19" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
-      <c r="J20">
-        <v>21002</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>14</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C21" s="1">
-        <v>2</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E21" s="1">
-        <v>0</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="E21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
-      <c r="J21">
-        <v>21003</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C22" s="1">
-        <v>2</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E22" s="1">
-        <v>0</v>
-      </c>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22">
-        <v>21004</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="13"/>
+      <c r="M22" s="13"/>
+      <c r="N22" s="13"/>
+      <c r="O22" s="13"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>28</v>
@@ -1419,12 +1427,12 @@
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23">
-        <v>21005</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+        <v>21001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>28</v>
@@ -1443,12 +1451,12 @@
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
       <c r="J24">
-        <v>21006</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+        <v>21002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>28</v>
@@ -1467,12 +1475,12 @@
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
       <c r="J25">
-        <v>21007</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+        <v>21003</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>28</v>
@@ -1491,12 +1499,12 @@
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26">
-        <v>21008</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+        <v>21004</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>28</v>
@@ -1515,12 +1523,12 @@
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
       <c r="J27">
-        <v>21009</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+        <v>21005</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>28</v>
@@ -1539,12 +1547,12 @@
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
       <c r="J28">
-        <v>21010</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+        <v>21006</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>28</v>
@@ -1563,12 +1571,12 @@
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
       <c r="J29">
-        <v>21011</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+        <v>21007</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>28</v>
@@ -1587,12 +1595,12 @@
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
       <c r="J30">
-        <v>21012</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+        <v>21008</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>28</v>
@@ -1611,12 +1619,12 @@
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
       <c r="J31">
-        <v>21013</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+        <v>21009</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>28</v>
@@ -1635,12 +1643,12 @@
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
       <c r="J32">
-        <v>21014</v>
+        <v>21010</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>28</v>
@@ -1659,12 +1667,12 @@
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
       <c r="J33">
-        <v>21015</v>
+        <v>21011</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>28</v>
@@ -1683,20 +1691,104 @@
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
       <c r="J34">
+        <v>21012</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>24</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C35" s="1">
+        <v>2</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E35" s="1">
+        <v>0</v>
+      </c>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35">
+        <v>21013</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>25</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C36" s="1">
+        <v>2</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E36" s="1">
+        <v>0</v>
+      </c>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+      <c r="J36">
+        <v>21014</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>26</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C37" s="1">
+        <v>2</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E37" s="1">
+        <v>0</v>
+      </c>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="1"/>
+      <c r="J37">
+        <v>21015</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>27</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C38" s="1">
+        <v>2</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E38" s="1">
+        <v>0</v>
+      </c>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1"/>
+      <c r="J38">
         <v>21016</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="E35" s="1"/>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="E36" s="1"/>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="E37" s="1"/>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="E38" s="1"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E39" s="1"/>
@@ -1715,11 +1807,23 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E44" s="1"/>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E45" s="1"/>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E46" s="1"/>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E47" s="1"/>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="E48" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
arranged item list spreadsheet
</commit_message>
<xml_diff>
--- a/assets/item_list.xlsx
+++ b/assets/item_list.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20361"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B1F75F8-BF87-43BC-9FAD-CADCC0932735}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ABF7E0E-FFF4-4E31-A8A2-5669F2D49D25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="76">
   <si>
     <t>halberd</t>
   </si>
@@ -170,21 +170,6 @@
     <t>Miscellaneous</t>
   </si>
   <si>
-    <t>Common</t>
-  </si>
-  <si>
-    <t>Uncommon</t>
-  </si>
-  <si>
-    <t>Rare</t>
-  </si>
-  <si>
-    <t>Epic</t>
-  </si>
-  <si>
-    <t>*rarity 1 and class type 0 for now</t>
-  </si>
-  <si>
     <t>Power</t>
   </si>
   <si>
@@ -236,34 +221,34 @@
     <t>Fighter</t>
   </si>
   <si>
-    <t>fighter</t>
-  </si>
-  <si>
-    <t>archer</t>
-  </si>
-  <si>
-    <t>tank</t>
-  </si>
-  <si>
-    <t>beserker</t>
-  </si>
-  <si>
-    <t>wizard</t>
-  </si>
-  <si>
-    <t>assasin</t>
-  </si>
-  <si>
-    <t>demon</t>
-  </si>
-  <si>
-    <t>necromancer</t>
-  </si>
-  <si>
-    <t>ARMORS</t>
-  </si>
-  <si>
-    <t>WEAPONS</t>
+    <t>SSS</t>
+  </si>
+  <si>
+    <t>Type No.</t>
+  </si>
+  <si>
+    <t>Rarity No.</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>Archer</t>
+  </si>
+  <si>
+    <t>Wizard</t>
+  </si>
+  <si>
+    <t>Tank</t>
+  </si>
+  <si>
+    <t>Berserker</t>
+  </si>
+  <si>
+    <t>Necromancer</t>
+  </si>
+  <si>
+    <t>Assassin</t>
   </si>
 </sst>
 </file>
@@ -313,7 +298,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -336,11 +321,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -361,14 +359,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -649,7 +654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" customWidth="1"/>
@@ -664,71 +669,91 @@
     <col min="14" max="14" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1"/>
-      <c r="F1"/>
-      <c r="G1"/>
-      <c r="H1"/>
-      <c r="I1"/>
-      <c r="J1"/>
-      <c r="K1"/>
-      <c r="L1"/>
-      <c r="M1"/>
-      <c r="N1"/>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="M2" s="3" t="s">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="N2" s="3" t="s">
-        <v>56</v>
+      <c r="E2" s="1">
+        <v>2</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G2" s="1">
+        <v>8</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I2" s="1">
+        <v>5</v>
+      </c>
+      <c r="J2" s="1">
+        <v>128500</v>
+      </c>
+      <c r="K2" s="1">
+        <v>10</v>
+      </c>
+      <c r="L2" s="1">
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>12</v>
@@ -737,25 +762,25 @@
         <v>1</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E3" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="G3" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I3" s="1">
-        <v>5</v>
-      </c>
-      <c r="J3">
-        <v>1585</v>
+        <v>4</v>
+      </c>
+      <c r="J3" s="1">
+        <v>161400</v>
       </c>
       <c r="K3" s="1">
         <v>10</v>
@@ -766,7 +791,7 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>12</v>
@@ -775,25 +800,25 @@
         <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E4" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G4" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I4" s="1">
-        <v>4</v>
-      </c>
-      <c r="J4">
-        <v>1114</v>
+        <v>7</v>
+      </c>
+      <c r="J4" s="1">
+        <v>166700</v>
       </c>
       <c r="K4" s="1">
         <v>10</v>
@@ -804,7 +829,7 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>12</v>
@@ -813,25 +838,25 @@
         <v>1</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E5" s="1">
+        <v>5</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G5" s="1">
+        <v>1</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E5" s="1">
-        <v>1</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="G5" s="1">
-        <v>1</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>76</v>
-      </c>
       <c r="I5" s="1">
-        <v>7</v>
-      </c>
-      <c r="J5">
-        <v>1117</v>
+        <v>8</v>
+      </c>
+      <c r="J5" s="1">
+        <v>151800</v>
       </c>
       <c r="K5" s="1">
         <v>10</v>
@@ -842,7 +867,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>12</v>
@@ -851,25 +876,25 @@
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="E6" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G6" s="1">
-        <v>1</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>77</v>
+        <v>2</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="I6" s="1">
-        <v>8</v>
-      </c>
-      <c r="J6">
-        <v>1218</v>
+        <v>0</v>
+      </c>
+      <c r="J6" s="1">
+        <v>162000</v>
       </c>
       <c r="K6" s="1">
         <v>10</v>
@@ -880,7 +905,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>12</v>
@@ -889,23 +914,25 @@
         <v>1</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="E7" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G7" s="1">
         <v>2</v>
       </c>
-      <c r="H7" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="I7" s="1"/>
-      <c r="J7">
-        <v>1120</v>
+      <c r="H7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="I7" s="1">
+        <v>3</v>
+      </c>
+      <c r="J7" s="1">
+        <v>152300</v>
       </c>
       <c r="K7" s="1">
         <v>10</v>
@@ -916,7 +943,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>12</v>
@@ -925,25 +952,25 @@
         <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E8" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>72</v>
       </c>
       <c r="G8" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I8" s="1">
-        <v>3</v>
-      </c>
-      <c r="J8">
-        <v>1223</v>
+        <v>5</v>
+      </c>
+      <c r="J8" s="1">
+        <v>144500</v>
       </c>
       <c r="K8" s="1">
         <v>10</v>
@@ -954,7 +981,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>12</v>
@@ -963,25 +990,25 @@
         <v>1</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E9" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>73</v>
       </c>
       <c r="G9" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="I9" s="1">
-        <v>5</v>
-      </c>
-      <c r="J9">
-        <v>1345</v>
+        <v>1</v>
+      </c>
+      <c r="J9" s="1">
+        <v>145100</v>
       </c>
       <c r="K9" s="1">
         <v>10</v>
@@ -992,7 +1019,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>12</v>
@@ -1001,25 +1028,25 @@
         <v>1</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="E10" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G10" s="1">
         <v>5</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="I10" s="1">
-        <v>1</v>
-      </c>
-      <c r="J10">
-        <v>1351</v>
+        <v>8</v>
+      </c>
+      <c r="J10" s="1">
+        <v>125800</v>
       </c>
       <c r="K10" s="1">
         <v>10</v>
@@ -1030,7 +1057,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>12</v>
@@ -1039,25 +1066,25 @@
         <v>1</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E11" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>74</v>
       </c>
       <c r="G11" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="I11" s="1">
         <v>8</v>
       </c>
-      <c r="J11">
-        <v>1558</v>
+      <c r="J11" s="1">
+        <v>136800</v>
       </c>
       <c r="K11" s="1">
         <v>10</v>
@@ -1068,7 +1095,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>12</v>
@@ -1077,25 +1104,25 @@
         <v>1</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="E12" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="G12" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="I12" s="1">
-        <v>8</v>
-      </c>
-      <c r="J12">
-        <v>1468</v>
+        <v>2</v>
+      </c>
+      <c r="J12" s="1">
+        <v>153200</v>
       </c>
       <c r="K12" s="1">
         <v>10</v>
@@ -1106,7 +1133,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>12</v>
@@ -1115,25 +1142,25 @@
         <v>1</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E13" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="G13" s="1">
         <v>3</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I13" s="1">
-        <v>2</v>
-      </c>
-      <c r="J13">
-        <v>1232</v>
+        <v>6</v>
+      </c>
+      <c r="J13" s="1">
+        <v>143600</v>
       </c>
       <c r="K13" s="1">
         <v>10</v>
@@ -1144,7 +1171,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>12</v>
@@ -1153,25 +1180,25 @@
         <v>1</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="E14" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>75</v>
       </c>
       <c r="G14" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="I14" s="1">
-        <v>6</v>
-      </c>
-      <c r="J14">
-        <v>1336</v>
+        <v>1</v>
+      </c>
+      <c r="J14" s="1">
+        <v>167100</v>
       </c>
       <c r="K14" s="1">
         <v>10</v>
@@ -1182,7 +1209,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>12</v>
@@ -1191,25 +1218,25 @@
         <v>1</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="E15" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G15" s="1">
         <v>7</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I15" s="1">
-        <v>1</v>
-      </c>
-      <c r="J15">
-        <v>1171</v>
+        <v>2</v>
+      </c>
+      <c r="J15" s="1">
+        <v>157200</v>
       </c>
       <c r="K15" s="1">
         <v>10</v>
@@ -1220,7 +1247,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>12</v>
@@ -1229,25 +1256,25 @@
         <v>1</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E16" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="G16" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="I16" s="1">
-        <v>2</v>
-      </c>
-      <c r="J16">
-        <v>1272</v>
+        <v>0</v>
+      </c>
+      <c r="J16" s="1">
+        <v>138000</v>
       </c>
       <c r="K16" s="1">
         <v>10</v>
@@ -1256,9 +1283,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>12</v>
@@ -1267,23 +1294,25 @@
         <v>1</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E17" s="1">
+        <v>3</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G17" s="1">
+        <v>5</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I17" s="1">
         <v>4</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="G17" s="1">
-        <v>8</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="I17" s="1"/>
-      <c r="J17">
-        <v>1480</v>
+      <c r="J17" s="1">
+        <v>135400</v>
       </c>
       <c r="K17" s="1">
         <v>10</v>
@@ -1292,9 +1321,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>12</v>
@@ -1303,25 +1332,25 @@
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="E18" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="G18" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I18" s="1">
-        <v>4</v>
-      </c>
-      <c r="J18">
-        <v>1454</v>
+        <v>7</v>
+      </c>
+      <c r="J18" s="1">
+        <v>161700</v>
       </c>
       <c r="K18" s="1">
         <v>10</v>
@@ -1330,85 +1359,97 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="C19" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E19" s="1">
-        <v>1</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="G19" s="1">
-        <v>1</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I19" s="1">
-        <v>7</v>
-      </c>
-      <c r="J19">
-        <v>1</v>
-      </c>
-      <c r="K19" s="1">
-        <v>10</v>
-      </c>
-      <c r="L19" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="E20" s="1"/>
+        <v>0</v>
+      </c>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="10"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" s="1">
+        <v>2</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E20" s="1">
+        <v>0</v>
+      </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J20" s="10"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>79</v>
-      </c>
-      <c r="E21" s="1"/>
+        <v>14</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="1">
+        <v>2</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E21" s="1">
+        <v>0</v>
+      </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="12"/>
-      <c r="I22" s="12"/>
-      <c r="J22" s="13"/>
-      <c r="K22" s="13"/>
-      <c r="L22" s="13"/>
-      <c r="M22" s="13"/>
-      <c r="N22" s="13"/>
-      <c r="O22" s="13"/>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J21" s="10"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" s="1">
+        <v>2</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E22" s="1">
+        <v>0</v>
+      </c>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="10"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>28</v>
@@ -1417,7 +1458,7 @@
         <v>2</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E23" s="1">
         <v>0</v>
@@ -1426,13 +1467,11 @@
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
-      <c r="J23">
-        <v>21001</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J23" s="10"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>28</v>
@@ -1441,7 +1480,7 @@
         <v>2</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E24" s="1">
         <v>0</v>
@@ -1450,13 +1489,11 @@
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
-      <c r="J24">
-        <v>21002</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J24" s="10"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>28</v>
@@ -1465,7 +1502,7 @@
         <v>2</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E25" s="1">
         <v>0</v>
@@ -1474,13 +1511,11 @@
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
-      <c r="J25">
-        <v>21003</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J25" s="10"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>28</v>
@@ -1489,7 +1524,7 @@
         <v>2</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E26" s="1">
         <v>0</v>
@@ -1498,13 +1533,11 @@
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
-      <c r="J26">
-        <v>21004</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J26" s="10"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>28</v>
@@ -1513,7 +1546,7 @@
         <v>2</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E27" s="1">
         <v>0</v>
@@ -1522,13 +1555,11 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
-      <c r="J27">
-        <v>21005</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J27" s="10"/>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>28</v>
@@ -1537,7 +1568,7 @@
         <v>2</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E28" s="1">
         <v>0</v>
@@ -1546,13 +1577,11 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
-      <c r="J28">
-        <v>21006</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J28" s="10"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>28</v>
@@ -1561,7 +1590,7 @@
         <v>2</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E29" s="1">
         <v>0</v>
@@ -1570,13 +1599,11 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
-      <c r="J29">
-        <v>21007</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J29" s="10"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>28</v>
@@ -1585,7 +1612,7 @@
         <v>2</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E30" s="1">
         <v>0</v>
@@ -1594,13 +1621,11 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
-      <c r="J30">
-        <v>21008</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J30" s="10"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>28</v>
@@ -1609,7 +1634,7 @@
         <v>2</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E31" s="1">
         <v>0</v>
@@ -1618,13 +1643,11 @@
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
-      <c r="J31">
-        <v>21009</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J31" s="10"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>28</v>
@@ -1633,7 +1656,7 @@
         <v>2</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E32" s="1">
         <v>0</v>
@@ -1642,13 +1665,11 @@
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
-      <c r="J32">
-        <v>21010</v>
-      </c>
+      <c r="J32" s="10"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>28</v>
@@ -1657,7 +1678,7 @@
         <v>2</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E33" s="1">
         <v>0</v>
@@ -1666,13 +1687,11 @@
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
-      <c r="J33">
-        <v>21011</v>
-      </c>
+      <c r="J33" s="10"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>28</v>
@@ -1681,7 +1700,7 @@
         <v>2</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E34" s="1">
         <v>0</v>
@@ -1690,105 +1709,19 @@
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
-      <c r="J34">
-        <v>21012</v>
-      </c>
+      <c r="J34" s="10"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>24</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C35" s="1">
-        <v>2</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E35" s="1">
-        <v>0</v>
-      </c>
-      <c r="F35" s="1"/>
-      <c r="G35" s="1"/>
-      <c r="H35" s="1"/>
-      <c r="I35" s="1"/>
-      <c r="J35">
-        <v>21013</v>
-      </c>
+      <c r="E35" s="1"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>25</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C36" s="1">
-        <v>2</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E36" s="1">
-        <v>0</v>
-      </c>
-      <c r="F36" s="1"/>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
-      <c r="I36" s="1"/>
-      <c r="J36">
-        <v>21014</v>
-      </c>
+      <c r="E36" s="1"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>26</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C37" s="1">
-        <v>2</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E37" s="1">
-        <v>0</v>
-      </c>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
-      <c r="I37" s="1"/>
-      <c r="J37">
-        <v>21015</v>
-      </c>
+      <c r="E37" s="1"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>27</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C38" s="1">
-        <v>2</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E38" s="1">
-        <v>0</v>
-      </c>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1"/>
-      <c r="H38" s="1"/>
-      <c r="I38" s="1"/>
-      <c r="J38">
-        <v>21016</v>
-      </c>
+      <c r="E38" s="1"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E39" s="1"/>
@@ -1807,18 +1740,6 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E44" s="1"/>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="E45" s="1"/>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="E46" s="1"/>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="E47" s="1"/>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="E48" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1829,19 +1750,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C316504E-A4CF-4FFE-BF92-734B59BDD790}">
-  <dimension ref="A2:D19"/>
+  <dimension ref="A2:F21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
     <col min="3" max="3" width="10.85546875" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
@@ -1851,11 +1773,17 @@
       <c r="C3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="14" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
@@ -1863,13 +1791,19 @@
         <v>1</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="D4" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+      <c r="D4" s="15">
+        <v>1</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="F4" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>28</v>
       </c>
@@ -1877,13 +1811,19 @@
         <v>2</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D5" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+      <c r="D5" s="15">
+        <v>2</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F5" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>46</v>
       </c>
@@ -1891,13 +1831,19 @@
         <v>3</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D6" s="5">
+        <v>62</v>
+      </c>
+      <c r="D6" s="15">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F6" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>47</v>
       </c>
@@ -1905,63 +1851,112 @@
         <v>4</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D7" s="5">
+        <v>61</v>
+      </c>
+      <c r="D7" s="15">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F7" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>48</v>
       </c>
       <c r="B8" s="5">
         <v>5</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="5"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="C8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="15">
+        <v>5</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F8" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="12"/>
+      <c r="B9" s="12"/>
+      <c r="C9" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="16">
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="E9" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="F9" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="12"/>
+      <c r="E10" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F10" s="5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="12"/>
+      <c r="E11" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11" s="5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="12"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixed spreadsheet and adjusted Item class code to match the excel file
</commit_message>
<xml_diff>
--- a/assets/item_list.xlsx
+++ b/assets/item_list.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ABF7E0E-FFF4-4E31-A8A2-5669F2D49D25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C7643A-5F09-4610-82C4-5160DDCDE4D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -359,7 +359,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -372,6 +371,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1379,7 +1381,9 @@
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="10"/>
+      <c r="J19" s="16">
+        <v>200000</v>
+      </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -1401,7 +1405,9 @@
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
-      <c r="J20" s="10"/>
+      <c r="J20" s="16">
+        <v>200001</v>
+      </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -1423,7 +1429,9 @@
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
-      <c r="J21" s="10"/>
+      <c r="J21" s="16">
+        <v>200002</v>
+      </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -1445,7 +1453,9 @@
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
-      <c r="J22" s="10"/>
+      <c r="J22" s="16">
+        <v>200003</v>
+      </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
@@ -1467,7 +1477,9 @@
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
-      <c r="J23" s="10"/>
+      <c r="J23" s="16">
+        <v>200004</v>
+      </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
@@ -1489,7 +1501,9 @@
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
-      <c r="J24" s="10"/>
+      <c r="J24" s="16">
+        <v>200005</v>
+      </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -1511,7 +1525,9 @@
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
-      <c r="J25" s="10"/>
+      <c r="J25" s="16">
+        <v>200006</v>
+      </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
@@ -1533,7 +1549,9 @@
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
-      <c r="J26" s="10"/>
+      <c r="J26" s="16">
+        <v>200007</v>
+      </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
@@ -1555,7 +1573,9 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
-      <c r="J27" s="10"/>
+      <c r="J27" s="16">
+        <v>200008</v>
+      </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
@@ -1577,7 +1597,9 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
-      <c r="J28" s="10"/>
+      <c r="J28" s="16">
+        <v>200009</v>
+      </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
@@ -1599,7 +1621,9 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
-      <c r="J29" s="10"/>
+      <c r="J29" s="16">
+        <v>200010</v>
+      </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
@@ -1621,7 +1645,9 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
-      <c r="J30" s="10"/>
+      <c r="J30" s="16">
+        <v>200011</v>
+      </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
@@ -1643,7 +1669,9 @@
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
-      <c r="J31" s="10"/>
+      <c r="J31" s="16">
+        <v>200012</v>
+      </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -1665,7 +1693,9 @@
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
-      <c r="J32" s="10"/>
+      <c r="J32" s="16">
+        <v>200013</v>
+      </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
@@ -1687,7 +1717,9 @@
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
-      <c r="J33" s="10"/>
+      <c r="J33" s="16">
+        <v>200014</v>
+      </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
@@ -1709,7 +1741,9 @@
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
-      <c r="J34" s="10"/>
+      <c r="J34" s="16">
+        <v>200015</v>
+      </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E35" s="1"/>
@@ -1773,7 +1807,7 @@
       <c r="C3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="13" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="6" t="s">
@@ -1793,10 +1827,10 @@
       <c r="C4" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D4" s="15">
-        <v>1</v>
-      </c>
-      <c r="E4" s="13" t="s">
+      <c r="D4" s="14">
+        <v>1</v>
+      </c>
+      <c r="E4" s="12" t="s">
         <v>65</v>
       </c>
       <c r="F4" s="5">
@@ -1813,7 +1847,7 @@
       <c r="C5" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="14">
         <v>2</v>
       </c>
       <c r="E5" s="4" t="s">
@@ -1833,7 +1867,7 @@
       <c r="C6" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="14">
         <v>3</v>
       </c>
       <c r="E6" s="4" t="s">
@@ -1853,7 +1887,7 @@
       <c r="C7" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="14">
         <v>4</v>
       </c>
       <c r="E7" s="4" t="s">
@@ -1873,7 +1907,7 @@
       <c r="C8" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="14">
         <v>5</v>
       </c>
       <c r="E8" s="4" t="s">
@@ -1884,12 +1918,12 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="11" t="s">
+      <c r="A9" s="11"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="15">
         <v>6</v>
       </c>
       <c r="E9" s="4" t="s">
@@ -1900,7 +1934,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="12"/>
+      <c r="A10" s="11"/>
       <c r="E10" s="4" t="s">
         <v>75</v>
       </c>
@@ -1909,7 +1943,7 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="12"/>
+      <c r="A11" s="11"/>
       <c r="E11" s="4" t="s">
         <v>64</v>
       </c>
@@ -1918,7 +1952,7 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="12"/>
+      <c r="A12" s="11"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">

</xml_diff>